<commit_message>
docs: version 2.33.0 - actualizacion integral de documentacion tecnica, manuales y version de la aplicacion
</commit_message>
<xml_diff>
--- a/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
+++ b/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
@@ -699,7 +699,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.32.0</t>
+          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.33.0</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.32.0</t>
+          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.33.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: version 2.34.0 - actualizacion integral de documentacion institucional, manuales tecnicos y de usuario
</commit_message>
<xml_diff>
--- a/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
+++ b/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
@@ -699,7 +699,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.33.0</t>
+          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.34.0</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.33.0</t>
+          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.34.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: version 2.35.0 - actualizacion integral de documentacion institucional, manuales tecnicos y de usuario
- Incremento de version a 2.35.0 en pubspec.yaml, README.md, documentacion institucional y scripts.
- Actualizacion de C3_Manual_Tecnico, C3_Manual_de_Usuario, C3_Plan_de_Sostenibilidad y C3_Documentacion_Tecnica_de_Transferencia.
- Recompilacion de documentos PDF oficiales y cronograma maestro en Excel.
</commit_message>
<xml_diff>
--- a/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
+++ b/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
@@ -699,7 +699,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.34.0</t>
+          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.35.0</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.34.0</t>
+          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.35.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: version 2.36.0 - actualizacion integral de documentacion institucional, manuales tecnicos y de usuario
- Incremento de version a 2.36.0 en pubspec.yaml, auth_wrapper.dart, legal_content.dart, preference_service.dart y README.md.
- Actualizacion de C3_Manual_Tecnico, C3_Manual_de_Usuario, C3_Plan_de_Sostenibilidad y C3_Documentacion_Tecnica_de_Transferencia.
- Documentacion de modularizacion arquitectonica (chat, reportes, recetas), transicion GPU 120 FPS (ContainerTransformCard), editor de tratamientos (EditarTratamientoPage), expansion tactil de calendario (CalendarExpandHandle), pipeline CI/CD y 194 pruebas automatizadas.
- Recompilacion de documentos PDF oficiales y cronograma maestro en Excel.
</commit_message>
<xml_diff>
--- a/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
+++ b/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
@@ -699,7 +699,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.35.0</t>
+          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.36.0</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.35.0</t>
+          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.36.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: version 2.37.0 - actualizacion integral de documentacion institucional, diapositivas oficiales C3 y manuales
- Incremento de version a 2.37.0 en pubspec.yaml, legal_content.dart, auth_wrapper.dart, preference_service.dart y README.md.
- Incorporacion de diapositivas oficiales de sustentacion en PowerPoint (.pptx) y PDF (.pdf), guia de defensa y script generador.
- Actualizacion de C3_Manual_Tecnico, C3_Manual_de_Usuario, C3_Plan_de_Sostenibilidad y C3_Documentacion_Tecnica_de_Transferencia.
- Recompilacion de documentos PDF institucionales oficiales y cronogramas en Excel.
</commit_message>
<xml_diff>
--- a/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
+++ b/documentos/Cronograma_de_Actividades_MediTime_2026.xlsx
@@ -699,7 +699,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.36.0</t>
+          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.37.0</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.36.0</t>
+          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.37.0</t>
         </is>
       </c>
     </row>

</xml_diff>